<commit_message>
The dashboard updates automatically with each run
</commit_message>
<xml_diff>
--- a/src/puzzleset.xlsx
+++ b/src/puzzleset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a91971/Desktop/CHESSPECKER/chess-trainer/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D10ABA-52D2-1E44-A6C7-843DB98FE42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA1D51D-C75B-4648-B2EB-5E5818743F1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28800" yWindow="-5640" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,7 +145,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -466,7 +466,7 @@
     <col min="6" max="6" width="12.5" style="4" customWidth="1"/>
     <col min="7" max="7" width="16.83203125" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>